<commit_message>
Make templates generic V0.2
Co-authored-by: wangyuanzhong <wangyuanzhong@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/competitive-analysis-templates/data/matrix-subjective.xlsx
+++ b/competitive-analysis-templates/data/matrix-subjective.xlsx
@@ -426,22 +426,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>对比项 \ 型号</t>
+          <t>维度 \ 对象</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Phantom X2</t>
+          <t>对象 A</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Nova Air</t>
+          <t>对象 B</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Prism Lite</t>
+          <t>对象 C</t>
         </is>
       </c>
     </row>
@@ -449,105 +449,105 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>item_a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>item_b</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>item_c</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>价格区间</t>
+          <t>维度一</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>¥6499 起</t>
+          <t>内容 A1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>¥5299 起</t>
+          <t>内容 B1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>¥3999 起</t>
+          <t>内容 C1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>主摄方案</t>
+          <t>维度二</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1" 云台主摄</t>
+          <t>内容 A2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>50MP 双层晶体管</t>
+          <t>内容 B2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>64MP 主摄</t>
+          <t>内容 C2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>端侧 AI</t>
+          <t>维度三</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NPU 12TOPS</t>
+          <t>内容 A3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>端云混合</t>
+          <t>内容 B3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>基础场景</t>
+          <t>内容 C3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>生态联动</t>
+          <t>维度四</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>全场景互联</t>
+          <t>内容 A4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>办公协同</t>
+          <t>内容 B4</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>轻量周边</t>
+          <t>内容 C4</t>
         </is>
       </c>
     </row>
@@ -566,9 +566,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,17 +579,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Phantom X2</t>
+          <t>对象 A</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Nova Air</t>
+          <t>对象 B</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Prism Lite</t>
+          <t>对象 C</t>
         </is>
       </c>
     </row>
@@ -597,39 +597,39 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>item_a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>item_b</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>item_c</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>价格区间</t>
+          <t>维度一</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>渠道价含标准套装。可写多段文案；空行分段显示为独立段落。</t>
+          <t>这里填写对象 A 在维度一的说明。</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>多存储梯度与捆绑服务差价。</t>
+          <t>这里填写对象 B 在维度一的说明。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>入门价位与成本控制取向。</t>
+          <t>这里填写对象 C 在维度一的说明。</t>
         </is>
       </c>
     </row>
@@ -639,33 +639,29 @@
           <t>（图路径）</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://picsum.photos/seed/techprice1/520/220</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>主摄方案</t>
+          <t>维度二</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大底云台模组，夜景与防抖均衡。</t>
+          <t>这里填写对象 A 在维度二的说明。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>弱光成像与算法侧协同方案。</t>
+          <t>这里填写对象 B 在维度二的说明。</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>主流价位影像取向与成片风格。</t>
+          <t>这里填写对象 C 在维度二的说明。</t>
         </is>
       </c>
     </row>
@@ -675,33 +671,29 @@
           <t>（图路径）</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://picsum.photos/seed/techcam1/520/240</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>端侧 AI</t>
+          <t>维度三</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>端侧推理与隐私边界下的能力边界。</t>
+          <t>这里填写对象 A 在维度三的说明。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>时延与离线覆盖的组合策略。</t>
+          <t>这里填写对象 B 在维度三的说明。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>覆盖日常智能助手与影像增强。</t>
+          <t>这里填写对象 C 在维度三的说明。</t>
         </is>
       </c>
     </row>
@@ -718,22 +710,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>生态联动</t>
+          <t>维度四</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>手表、耳机、车况等多设备联动。</t>
+          <t>这里填写对象 A 在维度四的说明。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>跨屏同步与会议场景配套。</t>
+          <t>这里填写对象 B 在维度四的说明。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>配件与第三方生态接入能力。</t>
+          <t>这里填写对象 C 在维度四的说明。</t>
         </is>
       </c>
     </row>

</xml_diff>